<commit_message>
Enhance SIMS-Core request format
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R245f30da920a4eed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rd7913ba2dda54c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rad8e8fc219834f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R056aad8fd4bd4e4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R73e821dd8bf64383"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rc68519ce1c054750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R030e28bec67c4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R480a5dad20ad44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R38a6b5cfaf02445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4008b98697194ecc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R71b95734be004760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R91897cbf040142b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R3096c2eb879c44f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R3ca9442de28a40c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R9c546ea41c5c41a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rb313f0c8de5d4186"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R0ae82ee61a394706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R5062d1c88f2d4a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rd6157735f40844b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R116015dc62b3427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R6873518884504eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rc143a6a512544d86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.0</x:v>
+        <x:v>v5.2.1</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10268,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.0</x:v>
+        <x:v>5.2.1</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Fetch fresh queries in Improvement Navi
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R91897cbf040142b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R3096c2eb879c44f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R3ca9442de28a40c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R9c546ea41c5c41a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rb313f0c8de5d4186"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R0ae82ee61a394706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R5062d1c88f2d4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rd6157735f40844b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R116015dc62b3427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R6873518884504eff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rc143a6a512544d86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Ra192b293eea349ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf2a9f2a6c83d472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rc654efd02d8d40a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R691daf6b8ad04276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R0b1933fd60e245ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R3cb527b0aff84c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R00beb4e88da647a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R4f43a316a8b74d0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R2fe53d418f914988"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rf78d8414ffcb45b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R273617054394460e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.1</x:v>
+        <x:v>v5.2.2</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10268,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.1</x:v>
+        <x:v>5.2.2</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Show query details in Improvement Navi
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Ra192b293eea349ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf2a9f2a6c83d472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rc654efd02d8d40a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R691daf6b8ad04276"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R0b1933fd60e245ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R3cb527b0aff84c28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R00beb4e88da647a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R4f43a316a8b74d0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R2fe53d418f914988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rf78d8414ffcb45b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R273617054394460e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rb455638c37694677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rbce33f808fa74bbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R3b2072f968fc412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R4404ba2ae66243f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rc06028c4c50b45b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Re5b53f0207e44d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R2cccaa5b77b448d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R8cbdb3b2058141ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R128dd230d8c246fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R2bc379cc09d14c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R9c663c209caa4d15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.2</x:v>
+        <x:v>v5.2.3</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10268,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.2</x:v>
+        <x:v>5.2.3</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Hide query sheet after Improvement Navi
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rb455638c37694677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rbce33f808fa74bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R3b2072f968fc412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R4404ba2ae66243f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rc06028c4c50b45b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Re5b53f0207e44d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R2cccaa5b77b448d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R8cbdb3b2058141ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R128dd230d8c246fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R2bc379cc09d14c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R9c663c209caa4d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Re5bdfd315e424555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf705cb3210b14d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rc73f554bbdc44e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Rcd65a9f7670643ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R7fc5f8160b344f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rd8751daf4390485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R27d0c74d1912441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R2b89d5ff46644508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Rbb77be666dec46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Re69327ca653c4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rd870ee11688c4861"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.3</x:v>
+        <x:v>v5.2.4</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10268,7 +10268,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.3</x:v>
+        <x:v>5.2.4</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Improve daily prompt and trend dates
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Re5bdfd315e424555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rf705cb3210b14d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rc73f554bbdc44e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Rcd65a9f7670643ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R7fc5f8160b344f22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rd8751daf4390485d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R27d0c74d1912441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R2b89d5ff46644508"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Rbb77be666dec46fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Re69327ca653c4709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rd870ee11688c4861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R97f0c725b8be4287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R2ae4cb3dcfa341b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rf832f598c84c4648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R2238e9c9e85141d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R29a3247c1ab74e91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rbfaaeb81d59841b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rb317737a4a084358"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R11181e3225da44ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R2db9bd046d9c4966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Ra58b483d876a4403"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R376890c59b234c38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.4</x:v>
+        <x:v>v5.2.5</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -6339,52 +6339,97 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="74" t="str">
+        <x:v>選択</x:v>
+      </x:c>
+      <x:c r="B1" s="74" t="str">
+        <x:v>改善実施日</x:v>
+      </x:c>
+      <x:c r="C1" s="74" t="str">
+        <x:v>経過日数</x:v>
+      </x:c>
+      <x:c r="D1" s="74" t="str">
+        <x:v>次回測定予定日</x:v>
+      </x:c>
+      <x:c r="E1" s="74" t="str">
+        <x:v>測定回数</x:v>
+      </x:c>
+      <x:c r="F1" s="74" t="str">
         <x:v>記事タイトル</x:v>
       </x:c>
-      <x:c r="B1" s="74" t="str">
-        <x:v>URL</x:v>
-      </x:c>
-      <x:c r="C1" s="74" t="str">
-        <x:v>改善日</x:v>
-      </x:c>
-      <x:c r="D1" s="74" t="str">
-        <x:v>改善内容</x:v>
-      </x:c>
-      <x:c r="E1" s="74" t="str">
-        <x:v>修正内容</x:v>
-      </x:c>
-      <x:c r="F1" s="74" t="str">
+      <x:c r="G1" s="74" t="str">
+        <x:v>改善前CTR</x:v>
+      </x:c>
+      <x:c r="H1" s="74" t="str">
+        <x:v>現在CTR</x:v>
+      </x:c>
+      <x:c r="I1" s="74" t="str">
         <x:v>改善前順位</x:v>
       </x:c>
-      <x:c r="G1" s="74" t="str">
+      <x:c r="J1" s="74" t="str">
         <x:v>現在順位</x:v>
       </x:c>
-      <x:c r="H1" s="74" t="str">
+      <x:c r="K1" s="74" t="str">
+        <x:v>判定</x:v>
+      </x:c>
+      <x:c r="L1" s="74" t="str">
+        <x:v>ArticleID</x:v>
+      </x:c>
+      <x:c r="M1" s="74" t="str">
+        <x:v>記事URL</x:v>
+      </x:c>
+      <x:c r="N1" s="74" t="str">
+        <x:v>改善概要</x:v>
+      </x:c>
+      <x:c r="O1" s="77" t="str">
+        <x:v>変更箇所</x:v>
+      </x:c>
+      <x:c r="P1" s="77" t="str">
+        <x:v>改善前クリック</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>現在クリック</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>クリック変化</x:v>
+      </x:c>
+      <x:c r="S1" t="str">
+        <x:v>改善前表示回数</x:v>
+      </x:c>
+      <x:c r="T1" t="str">
+        <x:v>現在表示回数</x:v>
+      </x:c>
+      <x:c r="U1" t="str">
+        <x:v>表示回数変化</x:v>
+      </x:c>
+      <x:c r="V1" t="str">
+        <x:v>CTR変化</x:v>
+      </x:c>
+      <x:c r="W1" t="str">
         <x:v>順位変化</x:v>
       </x:c>
-      <x:c r="I1" s="74" t="str">
-        <x:v>改善前CTR</x:v>
-      </x:c>
-      <x:c r="J1" s="74" t="str">
-        <x:v>現在CTR</x:v>
-      </x:c>
-      <x:c r="K1" s="74" t="str">
-        <x:v>CTR変化</x:v>
-      </x:c>
-      <x:c r="L1" s="74" t="str">
-        <x:v>改善前クリック</x:v>
-      </x:c>
-      <x:c r="M1" s="74" t="str">
-        <x:v>現在クリック</x:v>
-      </x:c>
-      <x:c r="N1" s="74" t="str">
-        <x:v>クリック変化</x:v>
-      </x:c>
-      <x:c r="O1" s="77" t="str">
-        <x:v>判定</x:v>
-      </x:c>
-      <x:c r="P1" s="77" t="str">
-        <x:v>コメント</x:v>
+      <x:c r="X1" t="str">
+        <x:v>期待CTR効果</x:v>
+      </x:c>
+      <x:c r="Y1" t="str">
+        <x:v>期待クリック効果</x:v>
+      </x:c>
+      <x:c r="Z1" t="str">
+        <x:v>SIMS評価</x:v>
+      </x:c>
+      <x:c r="AA1" t="str">
+        <x:v>次のアクション</x:v>
+      </x:c>
+      <x:c r="AB1" t="str">
+        <x:v>測定コメント</x:v>
+      </x:c>
+      <x:c r="AC1" t="str">
+        <x:v>最新測定日時</x:v>
+      </x:c>
+      <x:c r="AD1" t="str">
+        <x:v>測定状態</x:v>
+      </x:c>
+      <x:c r="AE1" t="str">
+        <x:v>改善履歴ID</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -10268,7 +10313,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.4</x:v>
+        <x:v>5.2.5</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Fix query retrieval and date displays
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R97f0c725b8be4287"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R2ae4cb3dcfa341b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rf832f598c84c4648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R2238e9c9e85141d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R29a3247c1ab74e91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rbfaaeb81d59841b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rb317737a4a084358"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R11181e3225da44ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R2db9bd046d9c4966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Ra58b483d876a4403"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R376890c59b234c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R889f597ea9664415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R67c21381eccb43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Re46426100daa44e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Raa1de4f7bfa84b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R47c8b8cb64e4476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R356344f5c5184c65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R82c6d992f62f4864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R918438a9ae9c4511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R66bc64ffbf164c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rd01076617cb34194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R44961019ddfc48ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,6 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy/M/d"/>
+  </x:numFmts>
   <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
@@ -357,7 +360,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="188">
+  <x:cellXfs count="189">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -859,6 +862,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="51" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1037,7 +1043,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.5</x:v>
+        <x:v>v5.2.6</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -6341,13 +6347,13 @@
       <x:c r="A1" s="74" t="str">
         <x:v>選択</x:v>
       </x:c>
-      <x:c r="B1" s="74" t="str">
+      <x:c r="B1" s="188" t="str">
         <x:v>改善実施日</x:v>
       </x:c>
       <x:c r="C1" s="74" t="str">
         <x:v>経過日数</x:v>
       </x:c>
-      <x:c r="D1" s="74" t="str">
+      <x:c r="D1" s="188" t="str">
         <x:v>次回測定予定日</x:v>
       </x:c>
       <x:c r="E1" s="74" t="str">
@@ -10313,7 +10319,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.5</x:v>
+        <x:v>5.2.6</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Reduce Improvement Navi query workload
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R889f597ea9664415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R67c21381eccb43c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Re46426100daa44e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Raa1de4f7bfa84b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R47c8b8cb64e4476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R356344f5c5184c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R82c6d992f62f4864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R918438a9ae9c4511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R66bc64ffbf164c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rd01076617cb34194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R44961019ddfc48ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R206c7b8f36044103"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R08721c4015a84845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R04400b5b8fb04184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Rae04edb68f4b43d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rb2f281bb67074664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Ree0f6abdbc934eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R1f27cc93d1f6467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R5357317ad90d4faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Rbb6be4c968ee4e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R197438c19a8f4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R3a5968ed5c6540cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -360,7 +360,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="189">
+  <x:cellXfs count="190">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -865,6 +865,9 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1043,7 +1046,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.6</x:v>
+        <x:v>v5.2.7</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -6353,7 +6356,7 @@
       <x:c r="C1" s="74" t="str">
         <x:v>経過日数</x:v>
       </x:c>
-      <x:c r="D1" s="188" t="str">
+      <x:c r="D1" s="189" t="str">
         <x:v>次回測定予定日</x:v>
       </x:c>
       <x:c r="E1" s="74" t="str">
@@ -10319,7 +10322,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.6</x:v>
+        <x:v>5.2.7</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Fix column references and corrupted details
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R206c7b8f36044103"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R08721c4015a84845"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R04400b5b8fb04184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Rae04edb68f4b43d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rb2f281bb67074664"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Ree0f6abdbc934eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R1f27cc93d1f6467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R5357317ad90d4faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Rbb6be4c968ee4e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R197438c19a8f4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R3a5968ed5c6540cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rb23c0931ac904f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R50a6c896a9b84ab1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R989992b5e7f844e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R75450c917f2e4fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R7dfa940b31904abd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Raeafde1a013548c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R8eab32302e64470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R25094f106dba4642"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R5e0165035663459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4e13d8058061451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R658fac7fd6a146cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1046,7 +1046,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.7</x:v>
+        <x:v>v5.2.8</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10322,7 +10322,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.7</x:v>
+        <x:v>5.2.8</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Clean invalid improvement history data
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rb23c0931ac904f9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R50a6c896a9b84ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R989992b5e7f844e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R75450c917f2e4fa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R7dfa940b31904abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Raeafde1a013548c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R8eab32302e64470c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R25094f106dba4642"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R5e0165035663459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4e13d8058061451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R658fac7fd6a146cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rd85b5ac779cb4158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R15e3d82f19a64e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Re23c3966f7634444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R04178b22ba274437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rf68f1a5017104a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R01b5d599b5e043d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R93ff9a32a6834839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rb98fbaeeb91247bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Re927dc7281e448a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R2b5ef01df3f844a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R2b415ca70aa449fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1046,7 +1046,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.8</x:v>
+        <x:v>v5.2.9</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10322,7 +10322,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.8</x:v>
+        <x:v>5.2.9</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>

<commit_message>
Stop orphan history rows returning
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.2-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rd85b5ac779cb4158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R15e3d82f19a64e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Re23c3966f7634444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R04178b22ba274437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="Rf68f1a5017104a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R01b5d599b5e043d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R93ff9a32a6834839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rb98fbaeeb91247bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Re927dc7281e448a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R2b5ef01df3f844a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R2b415ca70aa449fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R97099cdc525c497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R2b809dd893a54246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Raabc29bd9f414380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R54d59787c9014de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R4cf4675eeba34624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R291b70868fb24d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R591c05c59ae24827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R1261bc68629b4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Ra43a5d8c7a4d49ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4f9cf7abd0d842e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rd91b74e9c3f64c09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1046,7 +1046,7 @@
       <x:c r="F1" s="157"/>
       <x:c r="G1" s="157"/>
       <x:c r="H1" s="158" t="str">
-        <x:v>v5.2.9</x:v>
+        <x:v>v5.2.10</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -10322,7 +10322,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>5.2.9</x:v>
+        <x:v>5.2.10</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>

</xml_diff>